<commit_message>
Update analysis code and data to the latest version
Reorganize the analysis into shared helpers (functions.R) and
task-based scripts (meta_analysis.R, sensitivity.R, trends.R, maps.R,
descriptive.R, excluded_estimates.py, figures.py), replacing the
numbered scripts 00-14 and run_all.R.

Update review_data.xlsx and the study characteristics / quality score
workbook, add the B-lineage, case-control/test-negative and
mixed-design classification files, add requirements.txt and
.gitignore, and rewrite the README for the new layout.
</commit_message>
<xml_diff>
--- a/Data/Supplementary Data_Characteristics and Quality score.xlsx
+++ b/Data/Supplementary Data_Characteristics and Quality score.xlsx
@@ -1377,7 +1377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K352"/>
+  <dimension ref="A1:J352"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="28.283185840708" defaultRowHeight="17.6"/>
   <cols>
     <col width="12" customWidth="1" style="10" min="1" max="1"/>
@@ -1390,7 +1390,6 @@
     <col width="55" customWidth="1" style="10" min="8" max="8"/>
     <col width="22" customWidth="1" style="10" min="9" max="9"/>
     <col width="15" customWidth="1" style="10" min="10" max="10"/>
-    <col width="55" customWidth="1" style="10" min="11" max="11"/>
     <col width="28.283185840708" customWidth="1" style="11" min="12" max="16382"/>
     <col width="28.283185840708" customWidth="1" style="11" min="16383" max="16384"/>
   </cols>
@@ -1460,11 +1459,6 @@
           <t>Sample size</t>
         </is>
       </c>
-      <c r="K3" s="0" t="inlineStr">
-        <is>
-          <t>Source audit note</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="88.15000000000001" customHeight="1" s="30">
       <c r="A4" s="23" t="n">
@@ -3251,11 +3245,6 @@
       <c r="J42" s="29" t="n">
         <v>3841</v>
       </c>
-      <c r="K42" s="0" t="inlineStr">
-        <is>
-          <t>Includes 2015-16 estimates and legitimate pooled 2013-16 estimates.</t>
-        </is>
-      </c>
     </row>
     <row r="43" ht="52.9" customHeight="1" s="30">
       <c r="A43" s="23" t="n">
@@ -6652,11 +6641,6 @@
       <c r="J116" s="29" t="n">
         <v>610</v>
       </c>
-      <c r="K116" s="0" t="inlineStr">
-        <is>
-          <t>Effect table contains estimates for 2013-14, 2014-15, and 2015-16; earlier-season source citations should be listed with this study series.</t>
-        </is>
-      </c>
     </row>
     <row r="117" ht="52.9" customHeight="1" s="30">
       <c r="A117" s="23" t="n">
@@ -10527,7 +10511,7 @@
       </c>
       <c r="C201" s="29" t="inlineStr">
         <is>
-          <t>Suziki et al., 2014</t>
+          <t>Suzuki et al., 2014</t>
         </is>
       </c>
       <c r="D201" s="28" t="n">
@@ -11528,11 +11512,6 @@
       <c r="J222" s="23" t="n">
         <v>54434</v>
       </c>
-      <c r="K222" s="0" t="inlineStr">
-        <is>
-          <t>Original FOREVER analysis covers 2010-11 through 2015-16.</t>
-        </is>
-      </c>
     </row>
     <row r="223" ht="70.5" customFormat="1" customHeight="1" s="11">
       <c r="A223" s="23" t="n">
@@ -12143,7 +12122,7 @@
       </c>
       <c r="C236" s="23" t="inlineStr">
         <is>
-          <t>Palma-García et al. , 2025</t>
+          <t>Palma-García et al., 2025</t>
         </is>
       </c>
       <c r="D236" s="23" t="n">
@@ -14028,7 +14007,7 @@
       </c>
       <c r="C277" s="23" t="inlineStr">
         <is>
-          <t>McAnerne et al., 2015</t>
+          <t>McAnerney et al., 2015</t>
         </is>
       </c>
       <c r="D277" s="23" t="n">
@@ -16457,11 +16436,6 @@
       <c r="J329" s="23" t="n">
         <v>146662</v>
       </c>
-      <c r="K329" s="0" t="inlineStr">
-        <is>
-          <t>Corrected total study cohort; the VE analytic subset is 136,072. The old value 32,740 counted vaccinated participants only.</t>
-        </is>
-      </c>
     </row>
     <row r="330" ht="70.5" customHeight="1" s="30">
       <c r="A330" s="23" t="n">
@@ -17252,7 +17226,7 @@
       </c>
       <c r="C347" s="29" t="inlineStr">
         <is>
-          <t>Sturrman et al., 2020</t>
+          <t>Stuurman et al., 2020</t>
         </is>
       </c>
       <c r="D347" s="28" t="n">
@@ -17470,11 +17444,6 @@
       <c r="J351" s="29" t="n">
         <v>1441</v>
       </c>
-      <c r="K351" s="0" t="inlineStr">
-        <is>
-          <t>Article reports 2018-19, prior-season 2017-18, and pooled 2017-19 estimates.</t>
-        </is>
-      </c>
     </row>
     <row r="352" ht="70.5" customHeight="1" s="30">
       <c r="A352" s="23" t="n">
@@ -17525,7 +17494,7 @@
     <row r="353" ht="70.5" customHeight="1" s="30"/>
     <row r="354" ht="88.15000000000001" customHeight="1" s="30"/>
   </sheetData>
-  <autoFilter ref="A3:K352"/>
+  <autoFilter ref="A3:J352"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
@@ -20259,7 +20228,7 @@
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Arriola et al., 2019</t>
+          <t>Sofia Arriola et al., 2019</t>
         </is>
       </c>
       <c r="C72" s="11" t="n">
@@ -20335,7 +20304,7 @@
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>Kissling, et al., 2023</t>
+          <t>Kissling et al., 2023</t>
         </is>
       </c>
       <c r="C74" s="11" t="n">
@@ -20943,7 +20912,7 @@
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Blanchette et a.l, 2019</t>
+          <t>Blanchette et al., 2019</t>
         </is>
       </c>
       <c r="C90" s="11" t="n">
@@ -21741,7 +21710,7 @@
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Tenforde,et al., 2021</t>
+          <t>Tenforde et al., 2021</t>
         </is>
       </c>
       <c r="C111" s="11" t="n">
@@ -23071,7 +23040,7 @@
       </c>
       <c r="B146" s="11" t="inlineStr">
         <is>
-          <t>Gao et al., 2024</t>
+          <t>Gào et al., 2024</t>
         </is>
       </c>
       <c r="C146" s="11" t="n">
@@ -24439,7 +24408,7 @@
       </c>
       <c r="B182" s="11" t="inlineStr">
         <is>
-          <t>Suziki et al., 2014</t>
+          <t>Suzuki et al., 2014</t>
         </is>
       </c>
       <c r="C182" s="11" t="n">
@@ -25160,7 +25129,7 @@
       </c>
       <c r="B201" s="11" t="inlineStr">
         <is>
-          <t>Kuliese et al., 2021</t>
+          <t>Kuliese et al. , 2021</t>
         </is>
       </c>
       <c r="C201" s="11" t="n">
@@ -25234,7 +25203,7 @@
       </c>
       <c r="B203" s="11" t="inlineStr">
         <is>
-          <t>Choi et al., 2013</t>
+          <t>Choi et al. , 2013</t>
         </is>
       </c>
       <c r="C203" s="11" t="n">
@@ -26381,7 +26350,7 @@
       </c>
       <c r="B234" s="11" t="inlineStr">
         <is>
-          <t>Regan et al., 2025</t>
+          <t>Regan et al. , 2025</t>
         </is>
       </c>
       <c r="C234" s="11" t="n">
@@ -26418,7 +26387,7 @@
       </c>
       <c r="B235" s="11" t="inlineStr">
         <is>
-          <t>Chon et al., 2019</t>
+          <t>Chon et al. , 2019</t>
         </is>
       </c>
       <c r="C235" s="11" t="n">
@@ -27084,7 +27053,7 @@
       </c>
       <c r="B253" s="11" t="inlineStr">
         <is>
-          <t>McAnerne et al., 2015</t>
+          <t>McAnerney et al., 2015</t>
         </is>
       </c>
       <c r="C253" s="11" t="n">
@@ -29563,7 +29532,7 @@
       </c>
       <c r="B320" s="11" t="inlineStr">
         <is>
-          <t>Sturrman et al., 2020</t>
+          <t>Stuurman et al., 2020</t>
         </is>
       </c>
       <c r="C320" s="11" t="n">
@@ -30637,7 +30606,7 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Palma-García et al. , 2025</t>
+          <t>Palma-García et al., 2025</t>
         </is>
       </c>
       <c r="C23" s="11" t="n">

</xml_diff>